<commit_message>
(bugfix) [AC-448] : Removed duplicate services
</commit_message>
<xml_diff>
--- a/database/ddml-new/ServiceMapping.xlsx
+++ b/database/ddml-new/ServiceMapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kimoy\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SourceCloud\academically-app\database\ddml-new\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC7BBA7-996E-4998-BF46-1AFAD33B4433}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8109CF3D-D15C-40EB-AF34-86F5E03B0C0D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{DF9751C0-AC59-4711-8603-115DFB2F10A4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{DF9751C0-AC59-4711-8603-115DFB2F10A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="185">
   <si>
     <t>6c5e7af8-dd22-46d6-87b1-4436f2e4ab2f</t>
   </si>
@@ -178,18 +178,6 @@
     <t>Assessments Coaching</t>
   </si>
   <si>
-    <t>402410a6-d45f-423f-ab69-e62d55348dac</t>
-  </si>
-  <si>
-    <t>d76d644d-11b8-4f6a-8079-e7719e6a9c75</t>
-  </si>
-  <si>
-    <t>0c7b23af-c5a5-4e9d-8784-7994466a3a50</t>
-  </si>
-  <si>
-    <t>8c0821ff-9027-4177-b30c-17a6437b91cc</t>
-  </si>
-  <si>
     <t>CV Building</t>
   </si>
   <si>
@@ -208,75 +196,18 @@
     <t>Admissions Test Coaching</t>
   </si>
   <si>
-    <t>1b16ca5e-b334-4dff-aa6b-adb6e4ce89f1</t>
-  </si>
-  <si>
-    <t>4b4feede-0c51-4db2-b46a-4dc8abc4b7a8</t>
-  </si>
-  <si>
-    <t>b13d4c53-8b71-4f67-9912-0ab0d0714247</t>
-  </si>
-  <si>
     <t>fb25b847-c8d7-4185-b579-4def432a9c30</t>
   </si>
   <si>
     <t>Research Proposal Coaching</t>
   </si>
   <si>
-    <t>23a1dc9b-2e19-4edc-a2fa-5f2f741c3b79</t>
-  </si>
-  <si>
-    <t>a212df96-548c-4702-bba4-532e04494cbb</t>
-  </si>
-  <si>
-    <t>d07e3046-f681-4841-83eb-b7794c4e41d5</t>
-  </si>
-  <si>
-    <t>93cd7c91-e40f-459f-bd39-436d89221ca4</t>
-  </si>
-  <si>
-    <t>095dd7c5-ad35-430f-99ca-881b81468592</t>
-  </si>
-  <si>
-    <t>edc70fc2-c551-4f94-bfdf-93863da160ec</t>
-  </si>
-  <si>
-    <t>5ac68481-3c46-46f5-acd6-09be48dbafa8</t>
-  </si>
-  <si>
-    <t>41893412-8f67-4d58-baf2-abb4f96da0ba</t>
-  </si>
-  <si>
-    <t>d789a168-652b-49df-8367-0945e183486e</t>
-  </si>
-  <si>
-    <t>555381ae-f4fe-4b33-87ce-12e38f12ba6a</t>
-  </si>
-  <si>
-    <t>ef700f76-fbfc-475f-921b-bca9931f9719</t>
-  </si>
-  <si>
-    <t>1db2580e-8fe4-4c65-bf05-2af023676c02</t>
-  </si>
-  <si>
     <t>Academic Tutoring</t>
   </si>
   <si>
     <t>Assignment Feedback</t>
   </si>
   <si>
-    <t>57468258-b18a-47b8-b620-1a1af1d0d4a1</t>
-  </si>
-  <si>
-    <t>f47ee9ef-8c00-4008-b87f-69c778de0bd5</t>
-  </si>
-  <si>
-    <t>3fbed4b8-aa5e-4272-a264-4af14efd8edd</t>
-  </si>
-  <si>
-    <t>88b77771-9590-4f58-b04d-0d6ca75b6f05</t>
-  </si>
-  <si>
     <t>Proofreading &amp; Copy Editing</t>
   </si>
   <si>
@@ -544,21 +475,12 @@
     <t>Doctorate</t>
   </si>
   <si>
-    <t>24db2d03-c079-4619-bafb-26ad7d8ff261</t>
-  </si>
-  <si>
-    <t>b060591f-e4a8-4552-9903-0fbf41c6ed66</t>
-  </si>
-  <si>
     <t>359a60af-d41c-4aa2-8ce3-f1f3cee35c24</t>
   </si>
   <si>
     <t>Undergrad, Masters, Doctorate</t>
   </si>
   <si>
-    <t>f4c0dbdb-1144-431e-ae0f-f52fa4867703</t>
-  </si>
-  <si>
     <t>170485a2-6729-4b34-9375-43d0a756971f</t>
   </si>
   <si>
@@ -629,9 +551,6 @@
   </si>
   <si>
     <t>UK</t>
-  </si>
-  <si>
-    <t>79955c4b-f0a4-41f5-bedb-30a449b785a0</t>
   </si>
   <si>
     <t>4a37079a-5cce-4726-8cc9-e431940a0552</t>
@@ -716,554 +635,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="78">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1652,7 +1024,7 @@
         <v>672d3944-dd97-4a70-be11-fbc720d98645</v>
       </c>
       <c r="E4" t="s">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="F4" t="str">
         <f>VLOOKUP(E4,Services!$B$2:$C$118,2,0)</f>
@@ -1675,7 +1047,7 @@
         <v>2c3d46f8-ca19-4631-a47f-e808c4341a52</v>
       </c>
       <c r="E5" t="s">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="F5" t="str">
         <f>VLOOKUP(E5,Services!$B$2:$C$118,2,0)</f>
@@ -1698,7 +1070,7 @@
         <v>672d3944-dd97-4a70-be11-fbc720d98645</v>
       </c>
       <c r="E6" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="F6" t="str">
         <f>VLOOKUP(E6,Services!$B$2:$C$118,2,0)</f>
@@ -1721,7 +1093,7 @@
         <v>2c3d46f8-ca19-4631-a47f-e808c4341a52</v>
       </c>
       <c r="E7" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="F7" t="str">
         <f>VLOOKUP(E7,Services!$B$2:$C$118,2,0)</f>
@@ -1744,7 +1116,7 @@
         <v>672d3944-dd97-4a70-be11-fbc720d98645</v>
       </c>
       <c r="E8" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F8" t="str">
         <f>VLOOKUP(E8,Services!$B$2:$C$118,2,0)</f>
@@ -1767,7 +1139,7 @@
         <v>2c3d46f8-ca19-4631-a47f-e808c4341a52</v>
       </c>
       <c r="E9" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F9" t="str">
         <f>VLOOKUP(E9,Services!$B$2:$C$118,2,0)</f>
@@ -1783,7 +1155,7 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D10" t="str">
         <f>VLOOKUP(C10,Services!$B$2:$C$118,2,0)</f>
@@ -1803,7 +1175,7 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D11" t="str">
         <f>VLOOKUP(C11,Services!$B$2:$C$118,2,0)</f>
@@ -1823,7 +1195,7 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D12" t="str">
         <f>VLOOKUP(C12,Services!$B$2:$C$118,2,0)</f>
@@ -1843,7 +1215,7 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D13" t="str">
         <f>VLOOKUP(C13,Services!$B$2:$C$118,2,0)</f>
@@ -1863,7 +1235,7 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D14" t="str">
         <f>VLOOKUP(C14,Services!$B$2:$C$118,2,0)</f>
@@ -1883,7 +1255,7 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D15" t="str">
         <f>VLOOKUP(C15,Services!$B$2:$C$118,2,0)</f>
@@ -1923,14 +1295,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D17" t="str">
         <f>VLOOKUP(C17,Services!$B$2:$C$118,2,0)</f>
         <v>bcf7d458-6d6b-4c22-ae23-221acb81f24f</v>
       </c>
       <c r="E17" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F17" t="str">
         <f>VLOOKUP(E17,Services!$B$2:$C$118,2,0)</f>
@@ -1946,14 +1318,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D18" t="str">
         <f>VLOOKUP(C18,Services!$B$2:$C$118,2,0)</f>
         <v>1b7f6831-37f9-44e5-9fa9-8ee421061701</v>
       </c>
       <c r="E18" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F18" t="str">
         <f>VLOOKUP(E18,Services!$B$2:$C$118,2,0)</f>
@@ -1969,14 +1341,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D19" t="str">
         <f>VLOOKUP(C19,Services!$B$2:$C$118,2,0)</f>
         <v>be67df63-0749-4a39-9467-d2a0336db4b4</v>
       </c>
       <c r="E19" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F19" t="str">
         <f>VLOOKUP(E19,Services!$B$2:$C$118,2,0)</f>
@@ -1992,14 +1364,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D20" t="str">
         <f>VLOOKUP(C20,Services!$B$2:$C$118,2,0)</f>
         <v>8e9128d9-109d-4c8a-a758-ec6564d5ddbd</v>
       </c>
       <c r="E20" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F20" t="str">
         <f>VLOOKUP(E20,Services!$B$2:$C$118,2,0)</f>
@@ -2015,14 +1387,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D21" t="str">
         <f>VLOOKUP(C21,Services!$B$2:$C$118,2,0)</f>
         <v>9b62d92f-09ce-46b5-b09e-69136e867525</v>
       </c>
       <c r="E21" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F21" t="str">
         <f>VLOOKUP(E21,Services!$B$2:$C$118,2,0)</f>
@@ -2038,14 +1410,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C22" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D22" t="str">
         <f>VLOOKUP(C22,Services!$B$2:$C$118,2,0)</f>
         <v>3382a73a-885b-4191-a390-6f558c8912db</v>
       </c>
       <c r="E22" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F22" t="str">
         <f>VLOOKUP(E22,Services!$B$2:$C$118,2,0)</f>
@@ -2068,7 +1440,7 @@
         <v>2c3d46f8-ca19-4631-a47f-e808c4341a52</v>
       </c>
       <c r="E23" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="F23" t="str">
         <f>VLOOKUP(E23,Services!$B$2:$C$118,2,0)</f>
@@ -2084,14 +1456,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D24" t="str">
         <f>VLOOKUP(C24,Services!$B$2:$C$118,2,0)</f>
         <v>bcf7d458-6d6b-4c22-ae23-221acb81f24f</v>
       </c>
       <c r="E24" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F24" t="str">
         <f>VLOOKUP(E24,Services!$B$2:$C$118,2,0)</f>
@@ -2107,14 +1479,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D25" t="str">
         <f>VLOOKUP(C25,Services!$B$2:$C$118,2,0)</f>
         <v>1b7f6831-37f9-44e5-9fa9-8ee421061701</v>
       </c>
       <c r="E25" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F25" t="str">
         <f>VLOOKUP(E25,Services!$B$2:$C$118,2,0)</f>
@@ -2130,14 +1502,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C26" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D26" t="str">
         <f>VLOOKUP(C26,Services!$B$2:$C$118,2,0)</f>
         <v>be67df63-0749-4a39-9467-d2a0336db4b4</v>
       </c>
       <c r="E26" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F26" t="str">
         <f>VLOOKUP(E26,Services!$B$2:$C$118,2,0)</f>
@@ -2153,14 +1525,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D27" t="str">
         <f>VLOOKUP(C27,Services!$B$2:$C$118,2,0)</f>
         <v>8e9128d9-109d-4c8a-a758-ec6564d5ddbd</v>
       </c>
       <c r="E27" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F27" t="str">
         <f>VLOOKUP(E27,Services!$B$2:$C$118,2,0)</f>
@@ -2176,14 +1548,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D28" t="str">
         <f>VLOOKUP(C28,Services!$B$2:$C$118,2,0)</f>
         <v>9b62d92f-09ce-46b5-b09e-69136e867525</v>
       </c>
       <c r="E28" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F28" t="str">
         <f>VLOOKUP(E28,Services!$B$2:$C$118,2,0)</f>
@@ -2199,14 +1571,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D29" t="str">
         <f>VLOOKUP(C29,Services!$B$2:$C$118,2,0)</f>
         <v>3382a73a-885b-4191-a390-6f558c8912db</v>
       </c>
       <c r="E29" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F29" t="str">
         <f>VLOOKUP(E29,Services!$B$2:$C$118,2,0)</f>
@@ -2229,7 +1601,7 @@
         <v>2c3d46f8-ca19-4631-a47f-e808c4341a52</v>
       </c>
       <c r="E30" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="F30" t="str">
         <f>VLOOKUP(E30,Services!$B$2:$C$118,2,0)</f>
@@ -2245,14 +1617,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C31" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D31" t="str">
         <f>VLOOKUP(C31,Services!$B$2:$C$118,2,0)</f>
         <v>bcf7d458-6d6b-4c22-ae23-221acb81f24f</v>
       </c>
       <c r="E31" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F31" t="str">
         <f>VLOOKUP(E31,Services!$B$2:$C$118,2,0)</f>
@@ -2268,14 +1640,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C32" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D32" t="str">
         <f>VLOOKUP(C32,Services!$B$2:$C$118,2,0)</f>
         <v>1b7f6831-37f9-44e5-9fa9-8ee421061701</v>
       </c>
       <c r="E32" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F32" t="str">
         <f>VLOOKUP(E32,Services!$B$2:$C$118,2,0)</f>
@@ -2291,14 +1663,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D33" t="str">
         <f>VLOOKUP(C33,Services!$B$2:$C$118,2,0)</f>
         <v>be67df63-0749-4a39-9467-d2a0336db4b4</v>
       </c>
       <c r="E33" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F33" t="str">
         <f>VLOOKUP(E33,Services!$B$2:$C$118,2,0)</f>
@@ -2314,14 +1686,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C34" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D34" t="str">
         <f>VLOOKUP(C34,Services!$B$2:$C$118,2,0)</f>
         <v>8e9128d9-109d-4c8a-a758-ec6564d5ddbd</v>
       </c>
       <c r="E34" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F34" t="str">
         <f>VLOOKUP(E34,Services!$B$2:$C$118,2,0)</f>
@@ -2337,14 +1709,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C35" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D35" t="str">
         <f>VLOOKUP(C35,Services!$B$2:$C$118,2,0)</f>
         <v>9b62d92f-09ce-46b5-b09e-69136e867525</v>
       </c>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F35" t="str">
         <f>VLOOKUP(E35,Services!$B$2:$C$118,2,0)</f>
@@ -2360,14 +1732,14 @@
         <v>b4d0ce54-6fdc-4f8f-9265-7b56896bc2b1</v>
       </c>
       <c r="C36" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D36" t="str">
         <f>VLOOKUP(C36,Services!$B$2:$C$118,2,0)</f>
         <v>3382a73a-885b-4191-a390-6f558c8912db</v>
       </c>
       <c r="E36" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F36" t="str">
         <f>VLOOKUP(E36,Services!$B$2:$C$118,2,0)</f>
@@ -2390,7 +1762,7 @@
         <v>2c3d46f8-ca19-4631-a47f-e808c4341a52</v>
       </c>
       <c r="E37" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="F37" t="str">
         <f>VLOOKUP(E37,Services!$B$2:$C$118,2,0)</f>
@@ -2406,7 +1778,7 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C38" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="D38" t="str">
         <f>VLOOKUP(C38,Services!$B$2:$C$118,2,0)</f>
@@ -2426,7 +1798,7 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D39" t="str">
         <f>VLOOKUP(C39,Services!$B$2:$C$118,2,0)</f>
@@ -2446,7 +1818,7 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="D40" t="str">
         <f>VLOOKUP(C40,Services!$B$2:$C$118,2,0)</f>
@@ -2466,7 +1838,7 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C41" t="s">
-        <v>211</v>
+        <v>184</v>
       </c>
       <c r="D41" t="str">
         <f>VLOOKUP(C41,Services!$B$2:$C$118,2,0)</f>
@@ -2486,14 +1858,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="D42" t="str">
         <f>VLOOKUP(C42,Services!$B$2:$C$118,2,0)</f>
         <v>d20282ba-fbd3-4e72-81c0-3ec16309309c</v>
       </c>
       <c r="E42" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="F42" t="str">
         <f>VLOOKUP(E42,Services!$B$2:$C$118,2,0)</f>
@@ -2509,14 +1881,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D43" t="str">
         <f>VLOOKUP(C43,Services!$B$2:$C$118,2,0)</f>
         <v>90105083-583c-49b7-937e-22ce838591c0</v>
       </c>
       <c r="E43" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="F43" t="str">
         <f>VLOOKUP(E43,Services!$B$2:$C$118,2,0)</f>
@@ -2532,14 +1904,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C44" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="D44" t="str">
         <f>VLOOKUP(C44,Services!$B$2:$C$118,2,0)</f>
         <v>d20282ba-fbd3-4e72-81c0-3ec16309309c</v>
       </c>
       <c r="E44" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F44" t="str">
         <f>VLOOKUP(E44,Services!$B$2:$C$118,2,0)</f>
@@ -2555,14 +1927,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D45" t="str">
         <f>VLOOKUP(C45,Services!$B$2:$C$118,2,0)</f>
         <v>90105083-583c-49b7-937e-22ce838591c0</v>
       </c>
       <c r="E45" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F45" t="str">
         <f>VLOOKUP(E45,Services!$B$2:$C$118,2,0)</f>
@@ -2578,14 +1950,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C46" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="D46" t="str">
         <f>VLOOKUP(C46,Services!$B$2:$C$118,2,0)</f>
         <v>d20282ba-fbd3-4e72-81c0-3ec16309309c</v>
       </c>
       <c r="E46" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F46" t="str">
         <f>VLOOKUP(E46,Services!$B$2:$C$118,2,0)</f>
@@ -2601,14 +1973,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C47" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D47" t="str">
         <f>VLOOKUP(C47,Services!$B$2:$C$118,2,0)</f>
         <v>90105083-583c-49b7-937e-22ce838591c0</v>
       </c>
       <c r="E47" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F47" t="str">
         <f>VLOOKUP(E47,Services!$B$2:$C$118,2,0)</f>
@@ -2624,14 +1996,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C48" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="D48" t="str">
         <f>VLOOKUP(C48,Services!$B$2:$C$118,2,0)</f>
         <v>b0cd2298-822a-4515-9b61-4b4ee763bd98</v>
       </c>
       <c r="E48" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F48" t="str">
         <f>VLOOKUP(E48,Services!$B$2:$C$118,2,0)</f>
@@ -2647,14 +2019,14 @@
         <v>5065a4c4-9e2d-465b-b8a2-e3f1d89bfcc7</v>
       </c>
       <c r="C49" t="s">
-        <v>211</v>
+        <v>184</v>
       </c>
       <c r="D49" t="str">
         <f>VLOOKUP(C49,Services!$B$2:$C$118,2,0)</f>
         <v>263C4D7D-6AC7-4F4A-8B61-E6B3D72D9C5C</v>
       </c>
       <c r="E49" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F49" t="str">
         <f>VLOOKUP(E49,Services!$B$2:$C$118,2,0)</f>
@@ -2670,7 +2042,7 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="D50" t="str">
         <f>VLOOKUP(C50,Services!$B$2:$C$118,2,0)</f>
@@ -2690,7 +2062,7 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C51" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D51" t="str">
         <f>VLOOKUP(C51,Services!$B$2:$C$118,2,0)</f>
@@ -2710,7 +2082,7 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C52" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="D52" t="str">
         <f>VLOOKUP(C52,Services!$B$2:$C$118,2,0)</f>
@@ -2730,7 +2102,7 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C53" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="D53" t="str">
         <f>VLOOKUP(C53,Services!$B$2:$C$118,2,0)</f>
@@ -2750,7 +2122,7 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C54" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="D54" t="str">
         <f>VLOOKUP(C54,Services!$B$2:$C$118,2,0)</f>
@@ -2770,7 +2142,7 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C55" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="D55" t="str">
         <f>VLOOKUP(C55,Services!$B$2:$C$118,2,0)</f>
@@ -2790,14 +2162,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C56" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="D56" t="str">
         <f>VLOOKUP(C56,Services!$B$2:$C$118,2,0)</f>
         <v>9d268b81-efca-4334-b2b8-56abb0023b34</v>
       </c>
       <c r="E56" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="F56" t="str">
         <f>VLOOKUP(E56,Services!$B$2:$C$118,2,0)</f>
@@ -2813,14 +2185,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C57" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D57" t="str">
         <f>VLOOKUP(C57,Services!$B$2:$C$118,2,0)</f>
         <v>1bbc5625-9f81-4254-a9c4-94555c51f5da</v>
       </c>
       <c r="E57" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="F57" t="str">
         <f>VLOOKUP(E57,Services!$B$2:$C$118,2,0)</f>
@@ -2836,14 +2208,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="D58" t="str">
         <f>VLOOKUP(C58,Services!$B$2:$C$118,2,0)</f>
         <v>9d268b81-efca-4334-b2b8-56abb0023b34</v>
       </c>
       <c r="E58" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F58" t="str">
         <f>VLOOKUP(E58,Services!$B$2:$C$118,2,0)</f>
@@ -2859,14 +2231,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C59" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D59" t="str">
         <f>VLOOKUP(C59,Services!$B$2:$C$118,2,0)</f>
         <v>1bbc5625-9f81-4254-a9c4-94555c51f5da</v>
       </c>
       <c r="E59" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F59" t="str">
         <f>VLOOKUP(E59,Services!$B$2:$C$118,2,0)</f>
@@ -2882,14 +2254,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C60" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="D60" t="str">
         <f>VLOOKUP(C60,Services!$B$2:$C$118,2,0)</f>
         <v>4cb54c77-66a7-43e9-98ae-3c44da59b04b</v>
       </c>
       <c r="E60" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F60" t="str">
         <f>VLOOKUP(E60,Services!$B$2:$C$118,2,0)</f>
@@ -2905,14 +2277,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C61" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="D61" t="str">
         <f>VLOOKUP(C61,Services!$B$2:$C$118,2,0)</f>
         <v>0748d482-e4d0-456d-b9cf-39113e54c370</v>
       </c>
       <c r="E61" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F61" t="str">
         <f>VLOOKUP(E61,Services!$B$2:$C$118,2,0)</f>
@@ -2928,14 +2300,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C62" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="D62" t="str">
         <f>VLOOKUP(C62,Services!$B$2:$C$118,2,0)</f>
         <v>292ad230-9af7-4eb9-b85a-f27158898ff0</v>
       </c>
       <c r="E62" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F62" t="str">
         <f>VLOOKUP(E62,Services!$B$2:$C$118,2,0)</f>
@@ -2951,14 +2323,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C63" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="D63" t="str">
         <f>VLOOKUP(C63,Services!$B$2:$C$118,2,0)</f>
         <v>0e517fc6-d25d-4486-85db-c7f5506f4f50</v>
       </c>
       <c r="E63" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="F63" t="str">
         <f>VLOOKUP(E63,Services!$B$2:$C$118,2,0)</f>
@@ -2974,14 +2346,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C64" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="D64" t="str">
         <f>VLOOKUP(C64,Services!$B$2:$C$118,2,0)</f>
         <v>9d268b81-efca-4334-b2b8-56abb0023b34</v>
       </c>
       <c r="E64" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F64" t="str">
         <f>VLOOKUP(E64,Services!$B$2:$C$118,2,0)</f>
@@ -2997,14 +2369,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C65" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D65" t="str">
         <f>VLOOKUP(C65,Services!$B$2:$C$118,2,0)</f>
         <v>1bbc5625-9f81-4254-a9c4-94555c51f5da</v>
       </c>
       <c r="E65" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F65" t="str">
         <f>VLOOKUP(E65,Services!$B$2:$C$118,2,0)</f>
@@ -3020,14 +2392,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C66" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="D66" t="str">
         <f>VLOOKUP(C66,Services!$B$2:$C$118,2,0)</f>
         <v>4cb54c77-66a7-43e9-98ae-3c44da59b04b</v>
       </c>
       <c r="E66" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F66" t="str">
         <f>VLOOKUP(E66,Services!$B$2:$C$118,2,0)</f>
@@ -3043,14 +2415,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C67" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="D67" t="str">
         <f>VLOOKUP(C67,Services!$B$2:$C$118,2,0)</f>
         <v>0748d482-e4d0-456d-b9cf-39113e54c370</v>
       </c>
       <c r="E67" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F67" t="str">
         <f>VLOOKUP(E67,Services!$B$2:$C$118,2,0)</f>
@@ -3066,14 +2438,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C68" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="D68" t="str">
         <f>VLOOKUP(C68,Services!$B$2:$C$118,2,0)</f>
         <v>292ad230-9af7-4eb9-b85a-f27158898ff0</v>
       </c>
       <c r="E68" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F68" t="str">
         <f>VLOOKUP(E68,Services!$B$2:$C$118,2,0)</f>
@@ -3089,14 +2461,14 @@
         <v>2261bfdb-0998-4644-aeae-6af562d3373d</v>
       </c>
       <c r="C69" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="D69" t="str">
         <f>VLOOKUP(C69,Services!$B$2:$C$118,2,0)</f>
         <v>0e517fc6-d25d-4486-85db-c7f5506f4f50</v>
       </c>
       <c r="E69" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F69" t="str">
         <f>VLOOKUP(E69,Services!$B$2:$C$118,2,0)</f>
@@ -3112,7 +2484,7 @@
         <v>24f25767-bc02-46e1-8587-325dd8c3f6a4</v>
       </c>
       <c r="C70" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="D70" t="str">
         <f>VLOOKUP(C70,Services!$B$2:$C$118,2,0)</f>
@@ -3132,7 +2504,7 @@
         <v>24f25767-bc02-46e1-8587-325dd8c3f6a4</v>
       </c>
       <c r="C71" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="D71" t="str">
         <f>VLOOKUP(C71,Services!$B$2:$C$118,2,0)</f>
@@ -3152,7 +2524,7 @@
         <v>24f25767-bc02-46e1-8587-325dd8c3f6a4</v>
       </c>
       <c r="C72" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="D72" t="str">
         <f>VLOOKUP(C72,Services!$B$2:$C$118,2,0)</f>
@@ -3172,7 +2544,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C73" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="D73" t="str">
         <f>VLOOKUP(C73,Services!$B$2:$C$118,2,0)</f>
@@ -3192,7 +2564,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C74" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="D74" t="str">
         <f>VLOOKUP(C74,Services!$B$2:$C$118,2,0)</f>
@@ -3212,7 +2584,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C75" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="D75" t="str">
         <f>VLOOKUP(C75,Services!$B$2:$C$118,2,0)</f>
@@ -3232,7 +2604,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C76" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="D76" t="str">
         <f>VLOOKUP(C76,Services!$B$2:$C$118,2,0)</f>
@@ -3252,7 +2624,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C77" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="D77" t="str">
         <f>VLOOKUP(C77,Services!$B$2:$C$118,2,0)</f>
@@ -3272,7 +2644,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C78" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="D78" t="str">
         <f>VLOOKUP(C78,Services!$B$2:$C$118,2,0)</f>
@@ -3292,7 +2664,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C79" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="D79" t="str">
         <f>VLOOKUP(C79,Services!$B$2:$C$118,2,0)</f>
@@ -3312,7 +2684,7 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C80" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D80" t="str">
         <f>VLOOKUP(C80,Services!$B$2:$C$118,2,0)</f>
@@ -3332,14 +2704,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C81" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="D81" t="str">
         <f>VLOOKUP(C81,Services!$B$2:$C$118,2,0)</f>
         <v>5d3a658f-fcb8-4651-aa05-d27e10364159</v>
       </c>
       <c r="E81" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="F81" t="str">
         <f>VLOOKUP(E81,Services!$B$2:$C$118,2,0)</f>
@@ -3355,14 +2727,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C82" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="D82" t="str">
         <f>VLOOKUP(C82,Services!$B$2:$C$118,2,0)</f>
         <v>aff4984a-911b-42c2-9543-d6ca31205ea1</v>
       </c>
       <c r="E82" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="F82" t="str">
         <f>VLOOKUP(E82,Services!$B$2:$C$118,2,0)</f>
@@ -3378,14 +2750,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C83" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="D83" t="str">
         <f>VLOOKUP(C83,Services!$B$2:$C$118,2,0)</f>
         <v>4df3491a-539d-4f59-be81-27b9386621bf</v>
       </c>
       <c r="E83" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="F83" t="str">
         <f>VLOOKUP(E83,Services!$B$2:$C$118,2,0)</f>
@@ -3401,14 +2773,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C84" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="D84" t="str">
         <f>VLOOKUP(C84,Services!$B$2:$C$118,2,0)</f>
         <v>bdc3c6f6-f9cb-491a-ad94-9f0bec8008bb</v>
       </c>
       <c r="E84" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="F84" t="str">
         <f>VLOOKUP(E84,Services!$B$2:$C$118,2,0)</f>
@@ -3424,14 +2796,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C85" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="D85" t="str">
         <f>VLOOKUP(C85,Services!$B$2:$C$118,2,0)</f>
         <v>f4665639-2b55-4235-a7e1-44e793487f67</v>
       </c>
       <c r="E85" t="s">
-        <v>178</v>
+        <v>152</v>
       </c>
       <c r="F85" t="str">
         <f>VLOOKUP(E85,Services!$B$2:$C$118,2,0)</f>
@@ -3447,14 +2819,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C86" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="D86" t="str">
         <f>VLOOKUP(C86,Services!$B$2:$C$118,2,0)</f>
         <v>cb5d0f43-4d27-479b-acf8-eb3d81487b74</v>
       </c>
       <c r="E86" t="s">
-        <v>180</v>
+        <v>154</v>
       </c>
       <c r="F86" t="str">
         <f>VLOOKUP(E86,Services!$B$2:$C$118,2,0)</f>
@@ -3470,14 +2842,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C87" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="D87" t="str">
         <f>VLOOKUP(C87,Services!$B$2:$C$118,2,0)</f>
         <v>53e59a9a-d9e4-47c8-b77c-330d3cd4393e</v>
       </c>
       <c r="E87" t="s">
-        <v>182</v>
+        <v>156</v>
       </c>
       <c r="F87" t="str">
         <f>VLOOKUP(E87,Services!$B$2:$C$118,2,0)</f>
@@ -3493,14 +2865,14 @@
         <v>3ed54d43-46fa-43ce-8994-d10fff8604a6</v>
       </c>
       <c r="C88" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D88" t="str">
         <f>VLOOKUP(C88,Services!$B$2:$C$118,2,0)</f>
         <v>1b825955-6d65-4efd-8da6-bc21b613d719</v>
       </c>
       <c r="E88" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="F88" t="str">
         <f>VLOOKUP(E88,Services!$B$2:$C$118,2,0)</f>
@@ -3516,7 +2888,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C89" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="D89" t="str">
         <f>VLOOKUP(C89,Services!$B$2:$C$118,2,0)</f>
@@ -3536,7 +2908,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C90" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="D90" t="str">
         <f>VLOOKUP(C90,Services!$B$2:$C$118,2,0)</f>
@@ -3556,7 +2928,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C91" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="D91" t="str">
         <f>VLOOKUP(C91,Services!$B$2:$C$118,2,0)</f>
@@ -3576,7 +2948,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C92" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="D92" t="str">
         <f>VLOOKUP(C92,Services!$B$2:$C$118,2,0)</f>
@@ -3596,7 +2968,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C93" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="D93" t="str">
         <f>VLOOKUP(C93,Services!$B$2:$C$118,2,0)</f>
@@ -3616,7 +2988,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C94" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="D94" t="str">
         <f>VLOOKUP(C94,Services!$B$2:$C$118,2,0)</f>
@@ -3636,7 +3008,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C95" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="D95" t="str">
         <f>VLOOKUP(C95,Services!$B$2:$C$118,2,0)</f>
@@ -3656,7 +3028,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C96" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="D96" t="str">
         <f>VLOOKUP(C96,Services!$B$2:$C$118,2,0)</f>
@@ -3676,7 +3048,7 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C97" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="D97" t="str">
         <f>VLOOKUP(C97,Services!$B$2:$C$118,2,0)</f>
@@ -3696,14 +3068,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C98" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="D98" t="str">
         <f>VLOOKUP(C98,Services!$B$2:$C$118,2,0)</f>
         <v>c8e08cf7-3821-475b-90c5-c56f70f5ba3d</v>
       </c>
       <c r="E98" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F98" t="str">
         <f>VLOOKUP(E98,Services!$B$2:$C$118,2,0)</f>
@@ -3719,14 +3091,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C99" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="D99" t="str">
         <f>VLOOKUP(C99,Services!$B$2:$C$118,2,0)</f>
         <v>f975a1fe-2a0c-497d-a96d-33273428ff3b</v>
       </c>
       <c r="E99" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F99" t="str">
         <f>VLOOKUP(E99,Services!$B$2:$C$118,2,0)</f>
@@ -3742,14 +3114,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C100" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="D100" t="str">
         <f>VLOOKUP(C100,Services!$B$2:$C$118,2,0)</f>
         <v>445c0526-e355-433a-96c7-90833a34e514</v>
       </c>
       <c r="E100" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F100" t="str">
         <f>VLOOKUP(E100,Services!$B$2:$C$118,2,0)</f>
@@ -3765,14 +3137,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C101" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="D101" t="str">
         <f>VLOOKUP(C101,Services!$B$2:$C$118,2,0)</f>
         <v>c9bee77e-6e57-4e14-b22a-3fba9fbc15a6</v>
       </c>
       <c r="E101" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F101" t="str">
         <f>VLOOKUP(E101,Services!$B$2:$C$118,2,0)</f>
@@ -3788,14 +3160,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C102" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="D102" t="str">
         <f>VLOOKUP(C102,Services!$B$2:$C$118,2,0)</f>
         <v>ec7a72ff-cc70-451b-9e9e-feaec480d463</v>
       </c>
       <c r="E102" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F102" t="str">
         <f>VLOOKUP(E102,Services!$B$2:$C$118,2,0)</f>
@@ -3811,14 +3183,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C103" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="D103" t="str">
         <f>VLOOKUP(C103,Services!$B$2:$C$118,2,0)</f>
         <v>74be4041-91de-494d-8188-a046e2e30ede</v>
       </c>
       <c r="E103" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F103" t="str">
         <f>VLOOKUP(E103,Services!$B$2:$C$118,2,0)</f>
@@ -3834,14 +3206,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C104" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="D104" t="str">
         <f>VLOOKUP(C104,Services!$B$2:$C$118,2,0)</f>
         <v>9f811946-f3c2-4564-b044-93e0ec754ecb</v>
       </c>
       <c r="E104" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F104" t="str">
         <f>VLOOKUP(E104,Services!$B$2:$C$118,2,0)</f>
@@ -3857,14 +3229,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C105" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="D105" t="str">
         <f>VLOOKUP(C105,Services!$B$2:$C$118,2,0)</f>
         <v>587fc44b-ea9e-4e34-9be2-b35d4fb2da61</v>
       </c>
       <c r="E105" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F105" t="str">
         <f>VLOOKUP(E105,Services!$B$2:$C$118,2,0)</f>
@@ -3880,14 +3252,14 @@
         <v>8327fd9d-47be-4b79-817c-8364e60cc2b7</v>
       </c>
       <c r="C106" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="D106" t="str">
         <f>VLOOKUP(C106,Services!$B$2:$C$118,2,0)</f>
         <v>534256a9-3aed-43f9-8770-747385736da9</v>
       </c>
       <c r="E106" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="F106" t="str">
         <f>VLOOKUP(E106,Services!$B$2:$C$118,2,0)</f>
@@ -3903,7 +3275,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C107" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="D107" t="str">
         <f>VLOOKUP(C107,Services!$B$2:$C$118,2,0)</f>
@@ -3923,7 +3295,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C108" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="D108" t="str">
         <f>VLOOKUP(C108,Services!$B$2:$C$118,2,0)</f>
@@ -3943,7 +3315,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C109" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="D109" t="str">
         <f>VLOOKUP(C109,Services!$B$2:$C$118,2,0)</f>
@@ -3963,7 +3335,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C110" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="D110" t="str">
         <f>VLOOKUP(C110,Services!$B$2:$C$118,2,0)</f>
@@ -3983,7 +3355,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C111" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
       <c r="D111" t="str">
         <f>VLOOKUP(C111,Services!$B$2:$C$118,2,0)</f>
@@ -4003,7 +3375,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C112" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="D112" t="str">
         <f>VLOOKUP(C112,Services!$B$2:$C$118,2,0)</f>
@@ -4023,7 +3395,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C113" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="D113" t="str">
         <f>VLOOKUP(C113,Services!$B$2:$C$118,2,0)</f>
@@ -4043,7 +3415,7 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C114" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="D114" t="str">
         <f>VLOOKUP(C114,Services!$B$2:$C$118,2,0)</f>
@@ -4063,14 +3435,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C115" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="D115" t="str">
         <f>VLOOKUP(C115,Services!$B$2:$C$118,2,0)</f>
         <v>21ee1d45-03b3-413a-81e9-58169ee27810</v>
       </c>
       <c r="E115" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F115" t="str">
         <f>VLOOKUP(E115,Services!$B$2:$C$118,2,0)</f>
@@ -4086,14 +3458,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C116" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="D116" t="str">
         <f>VLOOKUP(C116,Services!$B$2:$C$118,2,0)</f>
         <v>ffed73d4-8915-48c9-abd1-b0c582e9003d</v>
       </c>
       <c r="E116" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F116" t="str">
         <f>VLOOKUP(E116,Services!$B$2:$C$118,2,0)</f>
@@ -4109,14 +3481,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C117" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="D117" t="str">
         <f>VLOOKUP(C117,Services!$B$2:$C$118,2,0)</f>
         <v>b54ad3bd-1684-4e35-9ad8-97e93af2e346</v>
       </c>
       <c r="E117" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F117" t="str">
         <f>VLOOKUP(E117,Services!$B$2:$C$118,2,0)</f>
@@ -4132,14 +3504,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C118" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="D118" t="str">
         <f>VLOOKUP(C118,Services!$B$2:$C$118,2,0)</f>
         <v>2c067fed-34fe-4be5-a3cb-8b4b108c03b6</v>
       </c>
       <c r="E118" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F118" t="str">
         <f>VLOOKUP(E118,Services!$B$2:$C$118,2,0)</f>
@@ -4155,14 +3527,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C119" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
       <c r="D119" t="str">
         <f>VLOOKUP(C119,Services!$B$2:$C$118,2,0)</f>
         <v>01786e53-00c3-4944-8398-6c2971ae36c8</v>
       </c>
       <c r="E119" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F119" t="str">
         <f>VLOOKUP(E119,Services!$B$2:$C$118,2,0)</f>
@@ -4178,14 +3550,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C120" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="D120" t="str">
         <f>VLOOKUP(C120,Services!$B$2:$C$118,2,0)</f>
         <v>6d493cc6-6caf-4bef-b12e-cba97c24892f</v>
       </c>
       <c r="E120" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F120" t="str">
         <f>VLOOKUP(E120,Services!$B$2:$C$118,2,0)</f>
@@ -4201,14 +3573,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C121" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="D121" t="str">
         <f>VLOOKUP(C121,Services!$B$2:$C$118,2,0)</f>
         <v>e1663fbd-7fa2-4ccb-a813-74606762fd49</v>
       </c>
       <c r="E121" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F121" t="str">
         <f>VLOOKUP(E121,Services!$B$2:$C$118,2,0)</f>
@@ -4224,14 +3596,14 @@
         <v>709a78df-a2b0-43c1-b7f3-3a354cfe8e7f</v>
       </c>
       <c r="C122" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="D122" t="str">
         <f>VLOOKUP(C122,Services!$B$2:$C$118,2,0)</f>
         <v>91a1ba4d-6e76-4114-b074-c9e8534b4de3</v>
       </c>
       <c r="E122" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F122" t="str">
         <f>VLOOKUP(E122,Services!$B$2:$C$118,2,0)</f>
@@ -4247,7 +3619,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C123" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="D123" t="str">
         <f>VLOOKUP(C123,Services!$B$2:$C$118,2,0)</f>
@@ -4267,7 +3639,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C124" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="D124" t="str">
         <f>VLOOKUP(C124,Services!$B$2:$C$118,2,0)</f>
@@ -4287,7 +3659,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C125" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="D125" t="str">
         <f>VLOOKUP(C125,Services!$B$2:$C$118,2,0)</f>
@@ -4307,7 +3679,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C126" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="D126" t="str">
         <f>VLOOKUP(C126,Services!$B$2:$C$118,2,0)</f>
@@ -4327,7 +3699,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C127" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="D127" t="str">
         <f>VLOOKUP(C127,Services!$B$2:$C$118,2,0)</f>
@@ -4347,7 +3719,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C128" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="D128" t="str">
         <f>VLOOKUP(C128,Services!$B$2:$C$118,2,0)</f>
@@ -4367,7 +3739,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C129" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="D129" t="str">
         <f>VLOOKUP(C129,Services!$B$2:$C$118,2,0)</f>
@@ -4387,7 +3759,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C130" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="D130" t="str">
         <f>VLOOKUP(C130,Services!$B$2:$C$118,2,0)</f>
@@ -4407,7 +3779,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C131" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="D131" t="str">
         <f>VLOOKUP(C131,Services!$B$2:$C$118,2,0)</f>
@@ -4427,7 +3799,7 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C132" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="D132" t="str">
         <f>VLOOKUP(C132,Services!$B$2:$C$118,2,0)</f>
@@ -4447,14 +3819,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C133" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="D133" t="str">
         <f>VLOOKUP(C133,Services!$B$2:$C$118,2,0)</f>
         <v>45edc2da-f829-4006-9cc5-652bdc0ac4c7</v>
       </c>
       <c r="E133" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F133" t="str">
         <f>VLOOKUP(E133,Services!$B$2:$C$118,2,0)</f>
@@ -4470,14 +3842,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C134" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="D134" t="str">
         <f>VLOOKUP(C134,Services!$B$2:$C$118,2,0)</f>
         <v>6ae2856f-08df-490d-ba9b-9bed26f55895</v>
       </c>
       <c r="E134" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F134" t="str">
         <f>VLOOKUP(E134,Services!$B$2:$C$118,2,0)</f>
@@ -4493,14 +3865,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C135" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="D135" t="str">
         <f>VLOOKUP(C135,Services!$B$2:$C$118,2,0)</f>
         <v>eb3e526c-8bd9-45af-a7ca-7ee1a879532c</v>
       </c>
       <c r="E135" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F135" t="str">
         <f>VLOOKUP(E135,Services!$B$2:$C$118,2,0)</f>
@@ -4516,14 +3888,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C136" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="D136" t="str">
         <f>VLOOKUP(C136,Services!$B$2:$C$118,2,0)</f>
         <v>477776b2-4a74-496e-944a-09130e2aaef1</v>
       </c>
       <c r="E136" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F136" t="str">
         <f>VLOOKUP(E136,Services!$B$2:$C$118,2,0)</f>
@@ -4539,14 +3911,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C137" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="D137" t="str">
         <f>VLOOKUP(C137,Services!$B$2:$C$118,2,0)</f>
         <v>03f3c5c0-0ad3-45b4-b4b7-87e2314514c1</v>
       </c>
       <c r="E137" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F137" t="str">
         <f>VLOOKUP(E137,Services!$B$2:$C$118,2,0)</f>
@@ -4562,14 +3934,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C138" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="D138" t="str">
         <f>VLOOKUP(C138,Services!$B$2:$C$118,2,0)</f>
         <v>45edc2da-f829-4006-9cc5-652bdc0ac4c7</v>
       </c>
       <c r="E138" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F138" t="str">
         <f>VLOOKUP(E138,Services!$B$2:$C$118,2,0)</f>
@@ -4585,14 +3957,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C139" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="D139" t="str">
         <f>VLOOKUP(C139,Services!$B$2:$C$118,2,0)</f>
         <v>6ae2856f-08df-490d-ba9b-9bed26f55895</v>
       </c>
       <c r="E139" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F139" t="str">
         <f>VLOOKUP(E139,Services!$B$2:$C$118,2,0)</f>
@@ -4608,14 +3980,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C140" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="D140" t="str">
         <f>VLOOKUP(C140,Services!$B$2:$C$118,2,0)</f>
         <v>eb3e526c-8bd9-45af-a7ca-7ee1a879532c</v>
       </c>
       <c r="E140" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F140" t="str">
         <f>VLOOKUP(E140,Services!$B$2:$C$118,2,0)</f>
@@ -4631,14 +4003,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C141" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="D141" t="str">
         <f>VLOOKUP(C141,Services!$B$2:$C$118,2,0)</f>
         <v>477776b2-4a74-496e-944a-09130e2aaef1</v>
       </c>
       <c r="E141" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F141" t="str">
         <f>VLOOKUP(E141,Services!$B$2:$C$118,2,0)</f>
@@ -4654,14 +4026,14 @@
         <v>76410084-1858-475b-a96c-87b4602daebc</v>
       </c>
       <c r="C142" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="D142" t="str">
         <f>VLOOKUP(C142,Services!$B$2:$C$118,2,0)</f>
         <v>03f3c5c0-0ad3-45b4-b4b7-87e2314514c1</v>
       </c>
       <c r="E142" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
       <c r="F142" t="str">
         <f>VLOOKUP(E142,Services!$B$2:$C$118,2,0)</f>
@@ -5825,7 +5197,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95BC6F5E-97C8-429D-8F65-DC1BCB97D6B8}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.42578125" customWidth="1"/>
@@ -5989,1146 +5361,849 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
         <v>46</v>
       </c>
-      <c r="B15" t="s">
-        <v>45</v>
-      </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
         <v>47</v>
       </c>
-      <c r="B16" t="s">
-        <v>13</v>
-      </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
         <v>48</v>
       </c>
-      <c r="B17" t="s">
-        <v>45</v>
-      </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
         <v>49</v>
       </c>
-      <c r="B18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" t="s">
-        <v>49</v>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
         <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>52</v>
       </c>
       <c r="B21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" t="s">
         <v>52</v>
       </c>
-      <c r="C21" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>10</v>
+      <c r="A22" t="s">
+        <v>18</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>10</v>
+        <v>54</v>
+      </c>
+      <c r="C22" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>61</v>
+      <c r="A29" s="1" t="s">
+        <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C29" t="s">
-        <v>61</v>
+        <v>66</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B30" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="C30" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B31" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="C32" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="B34" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B36" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>82</v>
       </c>
       <c r="C37" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="B39" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="C39" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="B40" t="s">
-        <v>13</v>
+        <v>88</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="B41" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>19</v>
+        <v>91</v>
       </c>
       <c r="B42" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C42" t="s">
-        <v>19</v>
+        <v>91</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="B43" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="C43" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="B44" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="C44" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="B46" t="s">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="C46" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>20</v>
+        <v>101</v>
       </c>
       <c r="B47" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="C47" t="s">
-        <v>20</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="C48" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="B49" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="C49" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="B50" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="C50" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="B51" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="C51" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
-        <v>88</v>
+      <c r="A52" t="s">
+        <v>111</v>
       </c>
       <c r="B52" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>88</v>
+        <v>112</v>
+      </c>
+      <c r="C52" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="C53" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="B54" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C54" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="B55" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="C55" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="C56" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="B57" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C57" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="B58" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="C58" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="B59" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="C59" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="B60" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="C60" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="B61" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="C61" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="B62" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="C62" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="B63" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="C63" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C64" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="B65" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="C65" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>3</v>
       </c>
       <c r="B66" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="C66" t="s">
-        <v>116</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>118</v>
+        <v>4</v>
       </c>
       <c r="B67" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="C67" t="s">
-        <v>118</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>120</v>
+        <v>5</v>
       </c>
       <c r="B68" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="C68" t="s">
-        <v>120</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="C69" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>124</v>
+        <v>15</v>
       </c>
       <c r="B70" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="C70" t="s">
-        <v>124</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>126</v>
+        <v>16</v>
       </c>
       <c r="B71" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="C71" t="s">
-        <v>126</v>
+        <v>16</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="B72" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="C72" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="B73" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="C73" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="B74" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="C74" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="B75" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="C75" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="B76" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="C76" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="B77" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="C77" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="B78" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="C78" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="B79" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="C79" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="B80" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="C80" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="B81" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="C81" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="B82" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="C82" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="B83" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="C83" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="B84" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="C84" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="B85" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="C85" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="B86" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="C86" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="B87" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="C87" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="B88" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="C88" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>3</v>
+        <v>179</v>
       </c>
       <c r="B89" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="C89" t="s">
-        <v>3</v>
+        <v>179</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>4</v>
+        <v>181</v>
       </c>
       <c r="B90" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="C90" t="s">
-        <v>4</v>
+        <v>181</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="B91" t="s">
-        <v>164</v>
+        <v>184</v>
       </c>
       <c r="C91" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>14</v>
-      </c>
-      <c r="B92" t="s">
-        <v>165</v>
-      </c>
-      <c r="C92" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>15</v>
-      </c>
-      <c r="B93" t="s">
-        <v>166</v>
-      </c>
-      <c r="C93" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>16</v>
-      </c>
-      <c r="B94" t="s">
-        <v>167</v>
-      </c>
-      <c r="C94" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>168</v>
-      </c>
-      <c r="B95" t="s">
-        <v>163</v>
-      </c>
-      <c r="C95" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>169</v>
-      </c>
-      <c r="B96" t="s">
-        <v>164</v>
-      </c>
-      <c r="C96" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>170</v>
-      </c>
-      <c r="B97" t="s">
-        <v>171</v>
-      </c>
-      <c r="C97" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>172</v>
-      </c>
-      <c r="B98" t="s">
-        <v>163</v>
-      </c>
-      <c r="C98" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>173</v>
-      </c>
-      <c r="B99" t="s">
-        <v>174</v>
-      </c>
-      <c r="C99" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>175</v>
-      </c>
-      <c r="B100" t="s">
-        <v>176</v>
-      </c>
-      <c r="C100" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>177</v>
-      </c>
-      <c r="B101" t="s">
-        <v>178</v>
-      </c>
-      <c r="C101" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>179</v>
-      </c>
-      <c r="B102" t="s">
-        <v>180</v>
-      </c>
-      <c r="C102" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>181</v>
-      </c>
-      <c r="B103" t="s">
-        <v>182</v>
-      </c>
-      <c r="C103" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
         <v>183</v>
-      </c>
-      <c r="B104" t="s">
-        <v>184</v>
-      </c>
-      <c r="C104" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>185</v>
-      </c>
-      <c r="B105" t="s">
-        <v>186</v>
-      </c>
-      <c r="C105" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>187</v>
-      </c>
-      <c r="B106" t="s">
-        <v>188</v>
-      </c>
-      <c r="C106" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>189</v>
-      </c>
-      <c r="B107" t="s">
-        <v>190</v>
-      </c>
-      <c r="C107" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>191</v>
-      </c>
-      <c r="B108" t="s">
-        <v>192</v>
-      </c>
-      <c r="C108" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>193</v>
-      </c>
-      <c r="B109" t="s">
-        <v>194</v>
-      </c>
-      <c r="C109" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>195</v>
-      </c>
-      <c r="B110" t="s">
-        <v>196</v>
-      </c>
-      <c r="C110" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>197</v>
-      </c>
-      <c r="B111" t="s">
-        <v>101</v>
-      </c>
-      <c r="C111" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>198</v>
-      </c>
-      <c r="B112" t="s">
-        <v>199</v>
-      </c>
-      <c r="C112" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>200</v>
-      </c>
-      <c r="B113" t="s">
-        <v>201</v>
-      </c>
-      <c r="C113" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>202</v>
-      </c>
-      <c r="B114" t="s">
-        <v>203</v>
-      </c>
-      <c r="C114" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>204</v>
-      </c>
-      <c r="B115" t="s">
-        <v>205</v>
-      </c>
-      <c r="C115" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>206</v>
-      </c>
-      <c r="B116" t="s">
-        <v>207</v>
-      </c>
-      <c r="C116" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>208</v>
-      </c>
-      <c r="B117" t="s">
-        <v>209</v>
-      </c>
-      <c r="C117" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>210</v>
-      </c>
-      <c r="B118" t="s">
-        <v>211</v>
-      </c>
-      <c r="C118" t="s">
-        <v>210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>